<commit_message>
Highlight fill-in price cells in red in prices_template.xlsx
</commit_message>
<xml_diff>
--- a/scripts/prices_template.xlsx
+++ b/scripts/prices_template.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,8 +28,11 @@
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <color rgb="00FF0000"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -39,6 +42,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00DDEBF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
   </fills>
@@ -54,11 +62,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -498,17 +507,16 @@
           <t>105g</t>
         </is>
       </c>
+      <c r="B3" s="2" t="n"/>
+      <c r="C3" s="2" t="n"/>
       <c r="D3" t="inlineStr">
         <is>
           <t>80g</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>230g</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr"/>
+      <c r="E3" s="2" t="n"/>
+      <c r="F3" s="2" t="n"/>
+      <c r="J3" s="2" t="n"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -516,16 +524,22 @@
           <t>128g</t>
         </is>
       </c>
+      <c r="B4" s="2" t="n"/>
+      <c r="C4" s="2" t="n"/>
       <c r="D4" t="inlineStr">
         <is>
           <t>100g</t>
         </is>
       </c>
+      <c r="E4" s="2" t="n"/>
+      <c r="F4" s="2" t="n"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>250g</t>
-        </is>
-      </c>
+          <t>230g</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="n"/>
+      <c r="I4" s="2" t="n"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -533,16 +547,22 @@
           <t>157g</t>
         </is>
       </c>
+      <c r="B5" s="2" t="n"/>
+      <c r="C5" s="2" t="n"/>
       <c r="D5" t="inlineStr">
         <is>
           <t>120g</t>
         </is>
       </c>
+      <c r="E5" s="2" t="n"/>
+      <c r="F5" s="2" t="n"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>300g</t>
-        </is>
-      </c>
+          <t>250g</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="n"/>
+      <c r="I5" s="2" t="n"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -550,6 +570,15 @@
           <t>200g</t>
         </is>
       </c>
+      <c r="B6" s="2" t="n"/>
+      <c r="C6" s="2" t="n"/>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>300g</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="n"/>
+      <c r="I6" s="2" t="n"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -557,17 +586,19 @@
           <t>250g</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="B7" s="2" t="n"/>
+      <c r="C7" s="2" t="n"/>
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t>骑马钉</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="E7" s="3" t="inlineStr">
         <is>
           <t>铜版胶钉A4</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="F7" s="3" t="inlineStr">
         <is>
           <t>胶版胶钉A4</t>
         </is>
@@ -579,21 +610,29 @@
           <t>300g</t>
         </is>
       </c>
+      <c r="B8" s="2" t="n"/>
+      <c r="C8" s="2" t="n"/>
+      <c r="D8" s="2" t="n"/>
+      <c r="E8" s="2" t="n"/>
+      <c r="F8" s="2" t="n"/>
     </row>
     <row r="9">
-      <c r="E9" s="2" t="inlineStr">
+      <c r="E9" s="3" t="inlineStr">
         <is>
           <t>覆膜（亮/哑/相膜）</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="F9" s="3" t="inlineStr">
         <is>
           <t>塑封A4</t>
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="E10" s="2" t="n"/>
+    </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>精装价格</t>
         </is>
@@ -632,6 +671,10 @@
           <t>锁线胶装</t>
         </is>
       </c>
+      <c r="C14" s="2" t="n"/>
+      <c r="E14" s="2" t="n"/>
+      <c r="F14" s="2" t="n"/>
+      <c r="G14" s="2" t="n"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -639,6 +682,10 @@
           <t>硬壳打钉精装</t>
         </is>
       </c>
+      <c r="C15" s="2" t="n"/>
+      <c r="E15" s="2" t="n"/>
+      <c r="F15" s="2" t="n"/>
+      <c r="G15" s="2" t="n"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -646,6 +693,10 @@
           <t>硬壳蝴蝶精装</t>
         </is>
       </c>
+      <c r="C16" s="2" t="n"/>
+      <c r="E16" s="2" t="n"/>
+      <c r="F16" s="2" t="n"/>
+      <c r="G16" s="2" t="n"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -653,6 +704,10 @@
           <t>硬壳锁线精装</t>
         </is>
       </c>
+      <c r="C17" s="2" t="n"/>
+      <c r="E17" s="2" t="n"/>
+      <c r="F17" s="2" t="n"/>
+      <c r="G17" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add self-paper double-side price column (K) to template and quote_xlsx.py
</commit_message>
<xml_diff>
--- a/scripts/prices_template.xlsx
+++ b/scripts/prices_template.xlsx
@@ -434,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:J17"/>
+  <dimension ref="A2:K17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -447,6 +447,7 @@
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -500,6 +501,11 @@
           <t>自带纸单面</t>
         </is>
       </c>
+      <c r="K2" s="1" t="inlineStr">
+        <is>
+          <t>自带纸双面</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -517,6 +523,7 @@
       <c r="E3" s="2" t="n"/>
       <c r="F3" s="2" t="n"/>
       <c r="J3" s="2" t="n"/>
+      <c r="K3" s="2" t="n"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">

</xml_diff>